<commit_message>
fix: navigation to SolarSystem3D screen and clean up dependencies
</commit_message>
<xml_diff>
--- a/automation/reports/test-results.xlsx
+++ b/automation/reports/test-results.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,12 +43,6 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
@@ -102,25 +96,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -488,14 +476,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="47" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
@@ -547,426 +535,6 @@
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Screenshot</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>TS_001</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>test_01_login_validation_errors</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>0.52s</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>TS_002</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>test_02_login_invalid_credentials</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>0.86s</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>TS_003</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>test_03_login_and_logout_cycle</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>1.34s</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>TS_004</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>test_04_sidebar_navigation</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>0.71s</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>TS_005</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>test_05_space_notes_ai_synthesis</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>1.25s</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>TS_006</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>test_06_space_chat_assistant</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>1.83s</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>TS_007</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>test_07_system_settings_control</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>2.03s</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>TS_008</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>test_08_launch_hub_schedule</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>0.92s</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>TS_009</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>test_09_satellite_radar_telemetry</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>0.89s</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>TS_010</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>test_10_unauthorized_direct_access_redirect</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>test_e2e_full</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Success / Passes Validation</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Verification Passed</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>0.18s</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1026,21 +594,21 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C4" s="6" t="n">
+      <c r="A4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="B4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -1179,49 +747,49 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>CHROME</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>150.0.7871.128</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Chrome</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Headless</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>3.12.6</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>4.22.0</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>09:08:26</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>09:10:17</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>111.35s</t>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>19:41:14</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>19:41:14</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>0.15s</t>
         </is>
       </c>
     </row>

</xml_diff>